<commit_message>
Fixing presence sheet back to french
</commit_message>
<xml_diff>
--- a/backend/src/templates/Consultant-template.xlsx
+++ b/backend/src/templates/Consultant-template.xlsx
@@ -2182,20 +2182,20 @@
     <mergeCell ref="B31:C31"/>
     <mergeCell ref="B32:C32"/>
     <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="C49:C50"/>
+    <mergeCell ref="B52:B54"/>
     <mergeCell ref="C52:C54"/>
-    <mergeCell ref="B52:B54"/>
-    <mergeCell ref="C49:C50"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="B43:C43"/>
-    <mergeCell ref="B42:C42"/>
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="B35:C35"/>
     <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B39:C39"/>
     <mergeCell ref="B40:C40"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B41:C41"/>
   </mergeCells>
   <printOptions/>
   <pageMargins bottom="0.35433070866141736" footer="0.0" header="0.0" left="0.5118110236220472" right="0.31496062992125984" top="0.35433070866141736"/>

</xml_diff>

<commit_message>
Fixing Presence sheet with signature V3
</commit_message>
<xml_diff>
--- a/backend/src/templates/Consultant-template.xlsx
+++ b/backend/src/templates/Consultant-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\excellia-app\backend\src\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4609C54-AC7D-4BF2-BC69-C553D64B5DD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{388379EC-2C9A-4352-AB57-BBFAA11147AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="50">
   <si>
     <t>Feuille de présence mission</t>
   </si>
@@ -164,9 +164,6 @@
   </si>
   <si>
     <t>Aymen Selmi</t>
-  </si>
-  <si>
-    <t>  Moez Dhehibi</t>
   </si>
   <si>
     <t>Date de signature</t>
@@ -289,7 +286,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="24">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -501,13 +498,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="FF9BBB59"/>
       </left>
@@ -576,7 +566,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -602,57 +592,38 @@
     <xf numFmtId="0" fontId="8" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -660,18 +631,31 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -695,9 +679,9 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>48</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>45720</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>99060</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="2743200" cy="1318260"/>
     <xdr:pic>
@@ -719,7 +703,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2293620" y="14813280"/>
+          <a:off x="2339340" y="15316200"/>
           <a:ext cx="2743200" cy="1318260"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -938,7 +922,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D997"/>
+  <dimension ref="A1:D996"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="33.44140625" customWidth="1"/>
@@ -952,12 +936,12 @@
       <c r="B1" s="1"/>
     </row>
     <row r="2" spans="1:4" ht="21" customHeight="1">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
     </row>
     <row r="3" spans="1:4" ht="14.25" customHeight="1"/>
     <row r="4" spans="1:4" ht="14.25" customHeight="1">
@@ -968,46 +952,46 @@
       <c r="A5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="35" t="s">
+      <c r="B5" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="29"/>
+      <c r="C5" s="17"/>
     </row>
     <row r="6" spans="1:4" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="36" t="s">
+      <c r="B6" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="29"/>
+      <c r="C6" s="17"/>
     </row>
     <row r="7" spans="1:4" ht="14.25" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="37" t="s">
+      <c r="B7" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="29"/>
+      <c r="C7" s="17"/>
     </row>
     <row r="8" spans="1:4" ht="14.25" customHeight="1">
       <c r="A8" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="36" t="s">
+      <c r="B8" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="29"/>
+      <c r="C8" s="17"/>
     </row>
     <row r="9" spans="1:4" ht="14.25" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="28" t="s">
+      <c r="B9" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="29"/>
+      <c r="C9" s="17"/>
     </row>
     <row r="10" spans="1:4" ht="14.25" customHeight="1">
       <c r="A10" s="1"/>
@@ -1021,10 +1005,10 @@
       <c r="A12" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="30" t="s">
+      <c r="B12" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="31"/>
+      <c r="C12" s="22"/>
       <c r="D12" s="5" t="s">
         <v>13</v>
       </c>
@@ -1033,10 +1017,10 @@
       <c r="A13" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="32" t="s">
-        <v>15</v>
-      </c>
-      <c r="C13" s="23"/>
+      <c r="B13" s="23" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" s="24"/>
       <c r="D13" s="7" t="s">
         <v>15</v>
       </c>
@@ -1045,10 +1029,10 @@
       <c r="A14" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="32" t="s">
-        <v>15</v>
-      </c>
-      <c r="C14" s="23"/>
+      <c r="B14" s="23" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="24"/>
       <c r="D14" s="7" t="s">
         <v>15</v>
       </c>
@@ -1057,10 +1041,10 @@
       <c r="A15" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="22" t="s">
-        <v>15</v>
-      </c>
-      <c r="C15" s="23"/>
+      <c r="B15" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C15" s="24"/>
       <c r="D15" s="8" t="s">
         <v>15</v>
       </c>
@@ -1069,10 +1053,10 @@
       <c r="A16" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="22" t="s">
-        <v>15</v>
-      </c>
-      <c r="C16" s="23"/>
+      <c r="B16" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C16" s="24"/>
       <c r="D16" s="8" t="s">
         <v>15</v>
       </c>
@@ -1081,10 +1065,10 @@
       <c r="A17" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="22" t="s">
-        <v>15</v>
-      </c>
-      <c r="C17" s="23"/>
+      <c r="B17" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17" s="24"/>
       <c r="D17" s="8" t="s">
         <v>15</v>
       </c>
@@ -1093,10 +1077,10 @@
       <c r="A18" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="22" t="s">
-        <v>15</v>
-      </c>
-      <c r="C18" s="23"/>
+      <c r="B18" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C18" s="24"/>
       <c r="D18" s="8" t="s">
         <v>15</v>
       </c>
@@ -1105,10 +1089,10 @@
       <c r="A19" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B19" s="22" t="s">
-        <v>15</v>
-      </c>
-      <c r="C19" s="23"/>
+      <c r="B19" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C19" s="24"/>
       <c r="D19" s="8" t="s">
         <v>15</v>
       </c>
@@ -1117,10 +1101,10 @@
       <c r="A20" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="22" t="s">
-        <v>15</v>
-      </c>
-      <c r="C20" s="23"/>
+      <c r="B20" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C20" s="24"/>
       <c r="D20" s="8" t="s">
         <v>15</v>
       </c>
@@ -1129,10 +1113,10 @@
       <c r="A21" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B21" s="22" t="s">
-        <v>15</v>
-      </c>
-      <c r="C21" s="23"/>
+      <c r="B21" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="24"/>
       <c r="D21" s="8" t="s">
         <v>15</v>
       </c>
@@ -1141,10 +1125,10 @@
       <c r="A22" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B22" s="22" t="s">
-        <v>15</v>
-      </c>
-      <c r="C22" s="23"/>
+      <c r="B22" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C22" s="24"/>
       <c r="D22" s="8" t="s">
         <v>15</v>
       </c>
@@ -1153,10 +1137,10 @@
       <c r="A23" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B23" s="22" t="s">
-        <v>15</v>
-      </c>
-      <c r="C23" s="23"/>
+      <c r="B23" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C23" s="24"/>
       <c r="D23" s="8" t="s">
         <v>15</v>
       </c>
@@ -1165,10 +1149,10 @@
       <c r="A24" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="22" t="s">
-        <v>15</v>
-      </c>
-      <c r="C24" s="23"/>
+      <c r="B24" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C24" s="24"/>
       <c r="D24" s="8" t="s">
         <v>15</v>
       </c>
@@ -1177,10 +1161,10 @@
       <c r="A25" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B25" s="22" t="s">
-        <v>15</v>
-      </c>
-      <c r="C25" s="23"/>
+      <c r="B25" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C25" s="24"/>
       <c r="D25" s="8" t="s">
         <v>15</v>
       </c>
@@ -1189,10 +1173,10 @@
       <c r="A26" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B26" s="22" t="s">
-        <v>15</v>
-      </c>
-      <c r="C26" s="23"/>
+      <c r="B26" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C26" s="24"/>
       <c r="D26" s="8" t="s">
         <v>15</v>
       </c>
@@ -1213,48 +1197,48 @@
       <c r="A28" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B28" s="24"/>
-      <c r="C28" s="21"/>
+      <c r="B28" s="28"/>
+      <c r="C28" s="29"/>
       <c r="D28" s="8"/>
     </row>
     <row r="29" spans="1:4" ht="30" customHeight="1">
       <c r="A29" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B29" s="24"/>
-      <c r="C29" s="21"/>
+      <c r="B29" s="28"/>
+      <c r="C29" s="29"/>
       <c r="D29" s="8"/>
     </row>
     <row r="30" spans="1:4" ht="30" customHeight="1">
       <c r="A30" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B30" s="24"/>
-      <c r="C30" s="21"/>
+      <c r="B30" s="28"/>
+      <c r="C30" s="29"/>
       <c r="D30" s="8"/>
     </row>
     <row r="31" spans="1:4" ht="30" customHeight="1">
       <c r="A31" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B31" s="24"/>
-      <c r="C31" s="21"/>
+      <c r="B31" s="28"/>
+      <c r="C31" s="29"/>
       <c r="D31" s="8"/>
     </row>
     <row r="32" spans="1:4" ht="30" customHeight="1">
       <c r="A32" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B32" s="24"/>
-      <c r="C32" s="21"/>
+      <c r="B32" s="28"/>
+      <c r="C32" s="29"/>
       <c r="D32" s="8"/>
     </row>
     <row r="33" spans="1:4" ht="30" customHeight="1">
       <c r="A33" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B33" s="24"/>
-      <c r="C33" s="21"/>
+      <c r="B33" s="28"/>
+      <c r="C33" s="29"/>
       <c r="D33" s="8" t="s">
         <v>15</v>
       </c>
@@ -1263,10 +1247,10 @@
       <c r="A34" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B34" s="20" t="s">
-        <v>15</v>
-      </c>
-      <c r="C34" s="21"/>
+      <c r="B34" s="35" t="s">
+        <v>15</v>
+      </c>
+      <c r="C34" s="29"/>
       <c r="D34" s="8" t="s">
         <v>15</v>
       </c>
@@ -1275,10 +1259,10 @@
       <c r="A35" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B35" s="22" t="s">
-        <v>15</v>
-      </c>
-      <c r="C35" s="23"/>
+      <c r="B35" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C35" s="24"/>
       <c r="D35" s="8" t="s">
         <v>15</v>
       </c>
@@ -1287,10 +1271,10 @@
       <c r="A36" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B36" s="22" t="s">
-        <v>15</v>
-      </c>
-      <c r="C36" s="23"/>
+      <c r="B36" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C36" s="24"/>
       <c r="D36" s="8" t="s">
         <v>15</v>
       </c>
@@ -1299,10 +1283,10 @@
       <c r="A37" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B37" s="22" t="s">
-        <v>15</v>
-      </c>
-      <c r="C37" s="23"/>
+      <c r="B37" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C37" s="24"/>
       <c r="D37" s="8" t="s">
         <v>15</v>
       </c>
@@ -1311,10 +1295,10 @@
       <c r="A38" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="B38" s="22" t="s">
-        <v>15</v>
-      </c>
-      <c r="C38" s="23"/>
+      <c r="B38" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C38" s="24"/>
       <c r="D38" s="8" t="s">
         <v>15</v>
       </c>
@@ -1323,10 +1307,10 @@
       <c r="A39" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="B39" s="22" t="s">
-        <v>15</v>
-      </c>
-      <c r="C39" s="23"/>
+      <c r="B39" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C39" s="24"/>
       <c r="D39" s="8" t="s">
         <v>15</v>
       </c>
@@ -1335,103 +1319,110 @@
       <c r="A40" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="B40" s="22" t="s">
-        <v>15</v>
-      </c>
-      <c r="C40" s="23"/>
+      <c r="B40" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C40" s="24"/>
       <c r="D40" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="30" customHeight="1">
-      <c r="A41" s="9"/>
-      <c r="B41" s="10" t="s">
+      <c r="A41" s="6"/>
+      <c r="B41" s="25"/>
+      <c r="C41" s="24"/>
+      <c r="D41" s="8"/>
+    </row>
+    <row r="42" spans="1:4" ht="30" customHeight="1">
+      <c r="A42" s="6"/>
+      <c r="B42" s="25"/>
+      <c r="C42" s="24"/>
+      <c r="D42" s="8"/>
+    </row>
+    <row r="43" spans="1:4" ht="20.399999999999999">
+      <c r="A43" s="6"/>
+      <c r="B43" s="25"/>
+      <c r="C43" s="24"/>
+      <c r="D43" s="8"/>
+    </row>
+    <row r="44" spans="1:4" ht="15" customHeight="1">
+      <c r="B44" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="C41" s="11">
+      <c r="C44" s="10">
         <v>0</v>
       </c>
-      <c r="D41" s="12"/>
-    </row>
-    <row r="42" spans="1:4" ht="30" customHeight="1">
-      <c r="A42" s="9"/>
-      <c r="B42" s="10" t="s">
+    </row>
+    <row r="45" spans="1:4" ht="15" customHeight="1">
+      <c r="B45" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="C42" s="11">
+      <c r="C45" s="10">
         <v>0</v>
       </c>
-      <c r="D42" s="12"/>
-    </row>
-    <row r="43" spans="1:4" ht="15" customHeight="1">
-      <c r="B43" s="13" t="s">
+    </row>
+    <row r="46" spans="1:4" ht="14.25" customHeight="1">
+      <c r="B46" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="C43" s="14" t="s">
+      <c r="C46" s="12" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="44" spans="1:4" ht="15" customHeight="1">
-      <c r="B44" s="15" t="s">
+    <row r="47" spans="1:4" ht="14.25" customHeight="1">
+      <c r="B47" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C44" s="15" t="s">
+      <c r="C47" s="13"/>
+    </row>
+    <row r="48" spans="1:4" ht="14.25" customHeight="1">
+      <c r="B48" s="11" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="45" spans="1:4" ht="15" customHeight="1">
-      <c r="B45" s="13" t="s">
+      <c r="C48" s="12" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="49" spans="2:3" ht="14.25" customHeight="1">
+      <c r="B49" s="30"/>
+      <c r="C49" s="30"/>
+    </row>
+    <row r="50" spans="2:3" ht="14.25" customHeight="1">
+      <c r="B50" s="31"/>
+      <c r="C50" s="31"/>
+    </row>
+    <row r="51" spans="2:3" ht="14.25" customHeight="1">
+      <c r="B51" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="C45" s="14" t="s">
+      <c r="C51" s="12" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="46" spans="1:4" ht="15" customHeight="1">
-      <c r="B46" s="25">
-        <v>46053</v>
-      </c>
-      <c r="C46" s="25"/>
-    </row>
-    <row r="47" spans="1:4" ht="14.25" customHeight="1">
-      <c r="B47" s="18"/>
-      <c r="C47" s="18"/>
-    </row>
-    <row r="48" spans="1:4" ht="14.25" customHeight="1">
-      <c r="B48" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="C48" s="14" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="49" spans="2:3" ht="14.25" customHeight="1">
-      <c r="B49" s="19"/>
-      <c r="C49" s="16"/>
-    </row>
-    <row r="50" spans="2:3" ht="14.25" customHeight="1">
-      <c r="B50" s="17"/>
-      <c r="C50" s="17"/>
-    </row>
-    <row r="51" spans="2:3" ht="14.25" customHeight="1">
-      <c r="B51" s="17"/>
-      <c r="C51" s="17"/>
-    </row>
     <row r="52" spans="2:3" ht="14.25" customHeight="1">
-      <c r="B52" s="17"/>
-      <c r="C52" s="17"/>
+      <c r="B52" s="34"/>
+      <c r="C52" s="32"/>
     </row>
     <row r="53" spans="2:3" ht="14.25" customHeight="1">
-      <c r="B53" s="17"/>
-      <c r="C53" s="17"/>
+      <c r="B53" s="33"/>
+      <c r="C53" s="33"/>
     </row>
     <row r="54" spans="2:3" ht="14.25" customHeight="1">
-      <c r="B54" s="18"/>
-      <c r="C54" s="18"/>
-    </row>
-    <row r="55" spans="2:3" ht="14.25" customHeight="1"/>
-    <row r="56" spans="2:3" ht="14.25" customHeight="1"/>
-    <row r="57" spans="2:3" ht="14.25" customHeight="1"/>
+      <c r="B54" s="33"/>
+      <c r="C54" s="33"/>
+    </row>
+    <row r="55" spans="2:3" ht="14.25" customHeight="1">
+      <c r="B55" s="33"/>
+      <c r="C55" s="33"/>
+    </row>
+    <row r="56" spans="2:3" ht="14.25" customHeight="1">
+      <c r="B56" s="33"/>
+      <c r="C56" s="33"/>
+    </row>
+    <row r="57" spans="2:3" ht="14.25" customHeight="1">
+      <c r="B57" s="31"/>
+      <c r="C57" s="31"/>
+    </row>
     <row r="58" spans="2:3" ht="14.25" customHeight="1"/>
     <row r="59" spans="2:3" ht="14.25" customHeight="1"/>
     <row r="60" spans="2:3" ht="14.25" customHeight="1"/>
@@ -1622,7 +1613,7 @@
     <row r="245" ht="14.25" customHeight="1"/>
     <row r="246" ht="14.25" customHeight="1"/>
     <row r="247" ht="14.25" customHeight="1"/>
-    <row r="248" ht="14.25" customHeight="1"/>
+    <row r="248" ht="15.75" customHeight="1"/>
     <row r="249" ht="15.75" customHeight="1"/>
     <row r="250" ht="15.75" customHeight="1"/>
     <row r="251" ht="15.75" customHeight="1"/>
@@ -2371,41 +2362,10 @@
     <row r="994" ht="15.75" customHeight="1"/>
     <row r="995" ht="15.75" customHeight="1"/>
     <row r="996" ht="15.75" customHeight="1"/>
-    <row r="997" ht="15.75" customHeight="1"/>
   </sheetData>
-  <mergeCells count="39">
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="C46:C47"/>
-    <mergeCell ref="C49:C54"/>
-    <mergeCell ref="B49:B54"/>
+  <mergeCells count="42">
+    <mergeCell ref="C52:C57"/>
+    <mergeCell ref="B52:B57"/>
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="B35:C35"/>
     <mergeCell ref="B36:C36"/>
@@ -2413,6 +2373,39 @@
     <mergeCell ref="B38:C38"/>
     <mergeCell ref="B39:C39"/>
     <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="C49:C50"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
   </mergeCells>
   <pageMargins left="0.51181102362204722" right="0.31496062992125984" top="0.35433070866141736" bottom="0.35433070866141736" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>